<commit_message>
updated the readings,simulations and plots of CC
</commit_message>
<xml_diff>
--- a/EXP_2/READINGS/CC_INPUT.xlsx
+++ b/EXP_2/READINGS/CC_INPUT.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EDC_LAB\EXP_2\READINGS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6E72E56-BD96-421A-A832-1B7BF255F49B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E92A7D9C-7631-4660-A915-49C2DC5BC341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C709E481-867C-4E09-872B-B4FEAFD754CF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{24D20B05-4044-4E22-A6B3-9EB1B8687072}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,18 +34,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
   <si>
-    <t>VBC</t>
+    <t>VCB</t>
   </si>
   <si>
-    <t>IB(uA)(VEC=1)</t>
+    <t>IB(uA)(VCE=1)</t>
   </si>
   <si>
-    <t>IB(uA)(VEC=5)</t>
+    <t>IB(uA)(VCE=5)</t>
   </si>
   <si>
-    <t>IB(uA)(VEC=10)</t>
+    <t>IB(uA)(VCE=10)</t>
   </si>
 </sst>
 </file>
@@ -159,7 +159,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>IB(uA)(VEC=1)</c:v>
+                  <c:v>IB(uA)(VCE=1)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -190,162 +190,114 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$25</c:f>
+              <c:f>Sheet1!$A$2:$A$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="24"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.26</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.05</c:v>
+                  <c:v>0.27</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1</c:v>
+                  <c:v>0.28999999999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.15</c:v>
+                  <c:v>0.31</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.2</c:v>
+                  <c:v>0.33</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.25</c:v>
+                  <c:v>0.35</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.3</c:v>
+                  <c:v>0.36</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.35</c:v>
+                  <c:v>0.37</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.4</c:v>
+                  <c:v>0.38</c:v>
                 </c:pt>
                 <c:pt idx="9">
+                  <c:v>0.39</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.41</c:v>
+                </c:pt>
+                <c:pt idx="11">
                   <c:v>0.42</c:v>
                 </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.44</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.46</c:v>
-                </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.48</c:v>
+                  <c:v>0.53</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.5</c:v>
+                  <c:v>0.55000000000000004</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.52</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.54</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0.56000000000000005</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0.57999999999999996</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>0.6</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0.62</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>0.64</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>0.66</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0.67999999999999905</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>0.69999999999999896</c:v>
+                  <c:v>0.97</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$B$2:$B$25</c:f>
+              <c:f>Sheet1!$B$2:$B$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="24"/>
+                <c:ptCount val="16"/>
                 <c:pt idx="0">
+                  <c:v>94</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>72.8</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>30.4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>21.9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>11.6</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6.3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>4.8</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>3.5</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.6</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="13">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.3</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.5</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>1.2</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>2.6</c:v>
-                </c:pt>
                 <c:pt idx="14">
-                  <c:v>4.4000000000000004</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>9.4</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>17.8</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>33.6</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>60</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>106.4</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>184.4</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>319.3</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>556.4</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>981.8</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -353,7 +305,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-49E0-4795-BA97-CB9595EDD97F}"/>
+              <c16:uniqueId val="{00000000-75FE-43B0-9737-671FFB23DCA5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -365,11 +317,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1754895983"/>
-        <c:axId val="1735876943"/>
+        <c:axId val="1468812160"/>
+        <c:axId val="1340818032"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1754895983"/>
+        <c:axId val="1468812160"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -426,12 +378,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1735876943"/>
+        <c:crossAx val="1340818032"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1735876943"/>
+        <c:axId val="1340818032"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -488,7 +440,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1754895983"/>
+        <c:crossAx val="1468812160"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -592,11 +544,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$C$1</c:f>
+              <c:f>Sheet1!$F$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>IB(uA)(VEC=5)</c:v>
+                  <c:v>IB(uA)(VCE=5)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -627,162 +579,84 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$25</c:f>
+              <c:f>Sheet1!$E$2:$E$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="24"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>4.3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.05</c:v>
+                  <c:v>4.32</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1</c:v>
+                  <c:v>4.34</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.15</c:v>
+                  <c:v>4.3600000000000003</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.2</c:v>
+                  <c:v>4.38</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.25</c:v>
+                  <c:v>4.4000000000000004</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.3</c:v>
+                  <c:v>4.42</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.35</c:v>
+                  <c:v>4.4400000000000004</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.4</c:v>
+                  <c:v>4.47</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.42</c:v>
+                  <c:v>4.5</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.44</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.46</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.48</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0.5</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0.52</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0.54</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>0.56000000000000005</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>0.57999999999999996</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>0.6</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>0.62</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>0.64</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>0.66</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>0.67999999999999905</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>0.69999999999999896</c:v>
+                  <c:v>4.8499999999999996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$C$2:$C$25</c:f>
+              <c:f>Sheet1!$F$2:$F$12</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="24"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>61.3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.1</c:v>
+                  <c:v>23.3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1</c:v>
+                  <c:v>9.3000000000000007</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1</c:v>
+                  <c:v>4.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.1</c:v>
+                  <c:v>2.2000000000000002</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.1</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.1</c:v>
+                  <c:v>0.4</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.3</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.5</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>1.2</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>2.6</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>4.4000000000000004</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>9.4</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>17.8</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>32.700000000000003</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>60</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>106.4</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>189.7</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>344.6</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>656.4</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>1625</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -790,7 +664,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D1CD-49F2-87E6-A1596FBDACA8}"/>
+              <c16:uniqueId val="{00000000-1C08-42B8-AA42-6520D35A2B5E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -802,11 +676,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1864386207"/>
-        <c:axId val="1735880783"/>
+        <c:axId val="1471142240"/>
+        <c:axId val="1340847792"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1864386207"/>
+        <c:axId val="1471142240"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -863,12 +737,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1735880783"/>
+        <c:crossAx val="1340847792"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1735880783"/>
+        <c:axId val="1340847792"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -925,7 +799,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1864386207"/>
+        <c:crossAx val="1471142240"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1029,11 +903,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$D$1</c:f>
+              <c:f>Sheet1!$J$1</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>IB(uA)(VEC=10)</c:v>
+                  <c:v>IB(uA)(VCE=10)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1064,114 +938,60 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$A$2:$A$17</c:f>
+              <c:f>Sheet1!$I$2:$I$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>9.34</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.05</c:v>
+                  <c:v>9.36</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1</c:v>
+                  <c:v>9.3800000000000008</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.15</c:v>
+                  <c:v>9.4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.2</c:v>
+                  <c:v>9.41</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.25</c:v>
+                  <c:v>9.42</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.3</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.35</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.4</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.42</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.44</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.46</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.48</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0.5</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>0.52</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0.54</c:v>
+                  <c:v>9.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$17</c:f>
+              <c:f>Sheet1!$J$2:$J$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>13.4</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5.0999999999999996</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.1</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.4</c:v>
+                </c:pt>
+                <c:pt idx="5">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0.1</c:v>
-                </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>0.2</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.3</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.5</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>0.8</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>1.9</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>4.4000000000000004</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1179,7 +999,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-D37E-46C4-8E79-F191FAAF8414}"/>
+              <c16:uniqueId val="{00000000-E715-4BD1-9E01-AB426502A6F8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1191,11 +1011,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1864431679"/>
-        <c:axId val="1735894703"/>
+        <c:axId val="1471147344"/>
+        <c:axId val="1340925552"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1864431679"/>
+        <c:axId val="1471147344"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1252,12 +1072,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1735894703"/>
+        <c:crossAx val="1340925552"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1735894703"/>
+        <c:axId val="1340925552"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1314,7 +1134,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1864431679"/>
+        <c:crossAx val="1471147344"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -3035,23 +2855,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>15240</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>179070</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>579120</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>320040</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>179070</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>274320</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>11430</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{40314365-361C-0923-27F1-99C76D230104}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F92F24BD-FAC1-DA91-6F1C-B7F2768313A7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3071,15 +2891,15 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>586740</xdr:colOff>
+      <xdr:row>18</xdr:row>
       <xdr:rowOff>3810</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>281940</xdr:colOff>
+      <xdr:row>33</xdr:row>
       <xdr:rowOff>3810</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3087,7 +2907,7 @@
         <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5E39EB6D-3E41-7230-4B96-64837B79FA7D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2FE5DCEC-0AF2-BE31-DAF5-66E2695B7DD8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3107,23 +2927,23 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>125730</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>15240</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>3810</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>125730</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>320040</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>3810</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="4" name="Chart 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{45359C8E-1732-C70F-666B-27D216B2CA10}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC0046A3-6C89-6686-42A9-E7E2F2485CB3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3440,334 +3260,264 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E9C6ADA8-85C0-45B4-B9D7-0DD68473FAD5}">
-  <dimension ref="A1:D25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08DEABFA-F611-4F91-9DD5-F45F2356DF68}">
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="I1" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2">
+        <v>0.26</v>
+      </c>
+      <c r="B2">
+        <v>94</v>
+      </c>
+      <c r="E2">
+        <v>4.3</v>
+      </c>
+      <c r="F2">
+        <v>61.3</v>
+      </c>
+      <c r="I2">
+        <v>9.34</v>
+      </c>
+      <c r="J2">
+        <v>13.4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>0.27</v>
+      </c>
+      <c r="B3">
+        <v>72.8</v>
+      </c>
+      <c r="E3">
+        <v>4.32</v>
+      </c>
+      <c r="F3">
+        <v>23.3</v>
+      </c>
+      <c r="I3">
+        <v>9.36</v>
+      </c>
+      <c r="J3">
+        <v>5.0999999999999996</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="B4">
+        <v>30.4</v>
+      </c>
+      <c r="E4">
+        <v>4.34</v>
+      </c>
+      <c r="F4">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="I4">
+        <v>9.3800000000000008</v>
+      </c>
+      <c r="J4">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>0.31</v>
+      </c>
+      <c r="B5">
+        <v>21.9</v>
+      </c>
+      <c r="E5">
+        <v>4.3600000000000003</v>
+      </c>
+      <c r="F5">
+        <v>4.5</v>
+      </c>
+      <c r="I5">
+        <v>9.4</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>0.33</v>
+      </c>
+      <c r="B6">
+        <v>11.6</v>
+      </c>
+      <c r="E6">
+        <v>4.38</v>
+      </c>
+      <c r="F6">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="I6">
+        <v>9.41</v>
+      </c>
+      <c r="J6">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>0.35</v>
+      </c>
+      <c r="B7">
+        <v>6.3</v>
+      </c>
+      <c r="E7">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>9.42</v>
+      </c>
+      <c r="J7">
         <v>0</v>
       </c>
-      <c r="B2">
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>0.36</v>
+      </c>
+      <c r="B8">
+        <v>4.8</v>
+      </c>
+      <c r="E8">
+        <v>4.42</v>
+      </c>
+      <c r="F8">
+        <v>0.4</v>
+      </c>
+      <c r="I8">
+        <v>9.5</v>
+      </c>
+      <c r="J8">
         <v>0</v>
       </c>
-      <c r="C2">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>0.37</v>
+      </c>
+      <c r="B9">
+        <v>3.5</v>
+      </c>
+      <c r="E9">
+        <v>4.4400000000000004</v>
+      </c>
+      <c r="F9">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>0.38</v>
+      </c>
+      <c r="B10">
+        <v>2.9</v>
+      </c>
+      <c r="E10">
+        <v>4.47</v>
+      </c>
+      <c r="F10">
         <v>0</v>
       </c>
-      <c r="D2">
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>0.39</v>
+      </c>
+      <c r="B11">
+        <v>1.6</v>
+      </c>
+      <c r="E11">
+        <v>4.5</v>
+      </c>
+      <c r="F11">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>0.05</v>
-      </c>
-      <c r="B3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>0.41</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>0.42</v>
+      </c>
+      <c r="B13">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>0.53</v>
+      </c>
+      <c r="B14">
         <v>0.1</v>
       </c>
-      <c r="C3">
-        <v>0.1</v>
-      </c>
-      <c r="D3">
-        <v>0.1</v>
-      </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>0.1</v>
-      </c>
-      <c r="B4">
-        <v>0.1</v>
-      </c>
-      <c r="C4">
-        <v>0.1</v>
-      </c>
-      <c r="D4">
-        <v>0.1</v>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>0.15</v>
-      </c>
-      <c r="B5">
-        <v>0.1</v>
-      </c>
-      <c r="C5">
-        <v>0.1</v>
-      </c>
-      <c r="D5">
-        <v>0.1</v>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>0.9</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>0.2</v>
-      </c>
-      <c r="B6">
-        <v>0.1</v>
-      </c>
-      <c r="C6">
-        <v>0.1</v>
-      </c>
-      <c r="D6">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>0.25</v>
-      </c>
-      <c r="B7">
-        <v>0.1</v>
-      </c>
-      <c r="C7">
-        <v>0.1</v>
-      </c>
-      <c r="D7">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>0.3</v>
-      </c>
-      <c r="B8">
-        <v>0.1</v>
-      </c>
-      <c r="C8">
-        <v>0.1</v>
-      </c>
-      <c r="D8">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>0.35</v>
-      </c>
-      <c r="B9">
-        <v>0.1</v>
-      </c>
-      <c r="C9">
-        <v>0.1</v>
-      </c>
-      <c r="D9">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>0.4</v>
-      </c>
-      <c r="B10">
-        <v>0.1</v>
-      </c>
-      <c r="C10">
-        <v>0.1</v>
-      </c>
-      <c r="D10">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>0.42</v>
-      </c>
-      <c r="B11">
-        <v>0.2</v>
-      </c>
-      <c r="C11">
-        <v>0.2</v>
-      </c>
-      <c r="D11">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12">
-        <v>0.44</v>
-      </c>
-      <c r="B12">
-        <v>0.3</v>
-      </c>
-      <c r="C12">
-        <v>0.3</v>
-      </c>
-      <c r="D12">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13">
-        <v>0.46</v>
-      </c>
-      <c r="B13">
-        <v>0.5</v>
-      </c>
-      <c r="C13">
-        <v>0.5</v>
-      </c>
-      <c r="D13">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14">
-        <v>0.48</v>
-      </c>
-      <c r="B14">
-        <v>1.2</v>
-      </c>
-      <c r="C14">
-        <v>1.2</v>
-      </c>
-      <c r="D14">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15">
-        <v>0.5</v>
-      </c>
-      <c r="B15">
-        <v>2.6</v>
-      </c>
-      <c r="C15">
-        <v>2.6</v>
-      </c>
-      <c r="D15">
-        <v>0.8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16">
-        <v>0.52</v>
-      </c>
-      <c r="B16">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="C16">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="D16">
-        <v>1.9</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>0.54</v>
+        <v>0.97</v>
       </c>
       <c r="B17">
-        <v>9.4</v>
-      </c>
-      <c r="C17">
-        <v>9.4</v>
-      </c>
-      <c r="D17">
-        <v>4.4000000000000004</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="B18">
-        <v>17.8</v>
-      </c>
-      <c r="C18">
-        <v>17.8</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="B19">
-        <v>33.6</v>
-      </c>
-      <c r="C19">
-        <v>32.700000000000003</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20">
-        <v>0.6</v>
-      </c>
-      <c r="B20">
-        <v>60</v>
-      </c>
-      <c r="C20">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21">
-        <v>0.62</v>
-      </c>
-      <c r="B21">
-        <v>106.4</v>
-      </c>
-      <c r="C21">
-        <v>106.4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22">
-        <v>0.64</v>
-      </c>
-      <c r="B22">
-        <v>184.4</v>
-      </c>
-      <c r="C22">
-        <v>189.7</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23">
-        <v>0.66</v>
-      </c>
-      <c r="B23">
-        <v>319.3</v>
-      </c>
-      <c r="C23">
-        <v>344.6</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24">
-        <v>0.67999999999999905</v>
-      </c>
-      <c r="B24">
-        <v>556.4</v>
-      </c>
-      <c r="C24">
-        <v>656.4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25">
-        <v>0.69999999999999896</v>
-      </c>
-      <c r="B25">
-        <v>981.8</v>
-      </c>
-      <c r="C25">
-        <v>1625</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>